<commit_message>
Update Tippmix data from web app
</commit_message>
<xml_diff>
--- a/tippmix.xlsx
+++ b/tippmix.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="294" uniqueCount="66">
   <si>
     <t>♠  TIPPMIX BANKROLL MANAGER  ♠</t>
   </si>
@@ -74,9 +74,6 @@
   </si>
   <si>
     <t>Veszített</t>
-  </si>
-  <si>
-    <t>Függőben</t>
   </si>
   <si>
     <t>♠  TIPPMIX – HAVI ELEMZÉS</t>
@@ -3354,7 +3351,7 @@
         <f>IF(OR(E73="",D73=""),"",E73*D73)</f>
       </c>
       <c r="G73" s="21" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="H73" s="20">
         <f>IF(G73="Nyert",F73,0)</f>
@@ -4181,7 +4178,7 @@
   <sheetData>
     <row r="1" ht="33.95" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -4193,22 +4190,22 @@
       <c r="I1"/>
       <c r="J1"/>
       <c r="L1" s="25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M1"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B3" s="27">
         <v>2026</v>
       </c>
       <c r="C3" s="28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="L3" s="29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="M3" s="30">
         <f>SUM(D7:D59)</f>
@@ -4224,7 +4221,7 @@
         <v>40</v>
       </c>
       <c r="N4" s="29" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O4" s="44">
         <f>SUM(H7:H59)</f>
@@ -4240,7 +4237,7 @@
         <v>26</v>
       </c>
       <c r="N5" s="29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O5" s="44">
         <f>SUM(I7:I59)</f>
@@ -4249,16 +4246,16 @@
     </row>
     <row r="6" ht="32.1" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="32" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" s="32" t="s">
         <v>34</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="C6" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="C6" s="32" t="s">
-        <v>36</v>
-      </c>
       <c r="D6" s="32" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E6" s="32" t="s">
         <v>14</v>
@@ -4267,26 +4264,26 @@
         <v>16</v>
       </c>
       <c r="G6" s="32" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="H6" s="32" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I6" s="32" t="s">
+        <v>29</v>
+      </c>
+      <c r="J6" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="J6" s="32" t="s">
-        <v>31</v>
-      </c>
       <c r="L6" s="29" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M6" s="33">
         <f>IFERROR(M4/M3,0)</f>
         <v>0.6060606060606061</v>
       </c>
       <c r="N6" s="29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O6" s="33">
         <f>IFERROR(O4/O5,0)</f>
@@ -6555,7 +6552,7 @@
   <sheetData>
     <row r="1" ht="26.25" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="47" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -6569,7 +6566,7 @@
     </row>
     <row r="3" ht="19.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="49" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B3" s="50">
         <f>SUM('Tippmix napló'!I7:I133)</f>
@@ -6580,7 +6577,7 @@
     </row>
     <row r="4" ht="19.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="49" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B4" s="50">
         <f>SUMIFS('Tippmix napló'!I7:I133,'Tippmix napló'!C7:C133,"&gt;="&amp;TODAY()-WEEKDAY(TODAY(),2)+1,'Tippmix napló'!C7:C133,"&lt;"&amp;TODAY()-WEEKDAY(TODAY(),2)+8)</f>
@@ -6591,7 +6588,7 @@
     </row>
     <row r="5" ht="19.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="49" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" s="50">
         <f>SUMIFS('Tippmix napló'!I7:I133,'Tippmix napló'!C7:C133,"&gt;="&amp;EOMONTH(TODAY(),-1)+1,'Tippmix napló'!C7:C133,"&lt;="&amp;EOMONTH(TODAY(),0))</f>
@@ -6602,7 +6599,7 @@
     </row>
     <row r="6" ht="19.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="49" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B6" s="51">
         <f>IFERROR(COUNTIF('Tippmix napló'!G7:G133,"Nyert")/(COUNTIF('Tippmix napló'!G7:G133,"Nyert")+COUNTIF('Tippmix napló'!G7:G133,"Veszített")),0)</f>
@@ -6613,7 +6610,7 @@
     </row>
     <row r="7" ht="19.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="49" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B7" s="51">
         <f>IFERROR(COUNTIFS('Tippmix napló'!G7:G133,"Nyert",'Tippmix napló'!C7:C133,"&gt;="&amp;TODAY()-WEEKDAY(TODAY(),2)+1,'Tippmix napló'!C7:C133,"&lt;"&amp;TODAY()-WEEKDAY(TODAY(),2)+8)/(COUNTIFS('Tippmix napló'!G7:G133,"Nyert",'Tippmix napló'!C7:C133,"&gt;="&amp;TODAY()-WEEKDAY(TODAY(),2)+1,'Tippmix napló'!C7:C133,"&lt;"&amp;TODAY()-WEEKDAY(TODAY(),2)+8)+COUNTIFS('Tippmix napló'!G7:G133,"Veszített",'Tippmix napló'!C7:C133,"&gt;="&amp;TODAY()-WEEKDAY(TODAY(),2)+1,'Tippmix napló'!C7:C133,"&lt;"&amp;TODAY()-WEEKDAY(TODAY(),2)+8)),0)</f>
@@ -6624,7 +6621,7 @@
     </row>
     <row r="8" ht="19.5" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="49" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B8" s="51">
         <f>IFERROR(COUNTIFS('Tippmix napló'!G7:G133,"Nyert",'Tippmix napló'!C7:C133,"&gt;="&amp;EOMONTH(TODAY(),-1)+1,'Tippmix napló'!C7:C133,"&lt;="&amp;EOMONTH(TODAY(),0))/(COUNTIFS('Tippmix napló'!G7:G133,"Nyert",'Tippmix napló'!C7:C133,"&gt;="&amp;EOMONTH(TODAY(),-1)+1,'Tippmix napló'!C7:C133,"&lt;="&amp;EOMONTH(TODAY(),0))+COUNTIFS('Tippmix napló'!G7:G133,"Veszített",'Tippmix napló'!C7:C133,"&gt;="&amp;EOMONTH(TODAY(),-1)+1,'Tippmix napló'!C7:C133,"&lt;="&amp;EOMONTH(TODAY(),0))),0)</f>
@@ -6665,7 +6662,7 @@
   <sheetData>
     <row r="1" ht="26.25" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -6683,13 +6680,13 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="52" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B3" s="53" t="s">
         <v>5</v>
       </c>
       <c r="C3" s="54" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D3"/>
       <c r="E3"/>
@@ -6697,13 +6694,13 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="52" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B4" s="53" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="54" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D4"/>
       <c r="E4"/>
@@ -6711,13 +6708,13 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="52" t="s">
+        <v>49</v>
+      </c>
+      <c r="B5" s="53" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="53" t="s">
+      <c r="C5" s="54" t="s">
         <v>51</v>
-      </c>
-      <c r="C5" s="54" t="s">
-        <v>52</v>
       </c>
       <c r="D5"/>
       <c r="E5"/>
@@ -6725,13 +6722,13 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="52" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B6" s="53" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="54" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D6"/>
       <c r="E6"/>
@@ -6739,13 +6736,13 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="52" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B7" s="53" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="54" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D7"/>
       <c r="E7"/>
@@ -6753,13 +6750,13 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="52" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B8" s="53" t="s">
         <v>9</v>
       </c>
       <c r="C8" s="54" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D8"/>
       <c r="E8"/>
@@ -6767,13 +6764,13 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="52" t="s">
+        <v>58</v>
+      </c>
+      <c r="B9" s="53" t="s">
         <v>59</v>
       </c>
-      <c r="B9" s="53" t="s">
+      <c r="C9" s="54" t="s">
         <v>60</v>
-      </c>
-      <c r="C9" s="54" t="s">
-        <v>61</v>
       </c>
       <c r="D9"/>
       <c r="E9"/>
@@ -6789,22 +6786,22 @@
     </row>
     <row r="12" ht="42" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="55" t="s">
+        <v>61</v>
+      </c>
+      <c r="B12" s="55" t="s">
         <v>62</v>
       </c>
-      <c r="B12" s="55" t="s">
+      <c r="C12" s="56" t="s">
         <v>63</v>
-      </c>
-      <c r="C12" s="56" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="13" ht="105" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="55"/>
       <c r="B13" s="55" t="s">
+        <v>64</v>
+      </c>
+      <c r="C13" s="56" t="s">
         <v>65</v>
-      </c>
-      <c r="C13" s="56" t="s">
-        <v>66</v>
       </c>
     </row>
   </sheetData>
@@ -6846,7 +6843,7 @@
   <sheetData>
     <row r="1" ht="33.95" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="24" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B1"/>
       <c r="C1"/>
@@ -6858,22 +6855,22 @@
       <c r="I1"/>
       <c r="J1"/>
       <c r="L1" s="25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M1"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="26" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B3" s="27">
         <v>2026</v>
       </c>
       <c r="C3" s="28" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" s="29" t="s">
         <v>21</v>
-      </c>
-      <c r="L3" s="29" t="s">
-        <v>22</v>
       </c>
       <c r="M3" s="30">
         <f>SUM(D7:D18)</f>
@@ -6889,7 +6886,7 @@
         <v>40</v>
       </c>
       <c r="N4" s="29" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="O4" s="31">
         <f>SUM(H7:H18)</f>
@@ -6905,7 +6902,7 @@
         <v>26</v>
       </c>
       <c r="N5" s="29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="O5" s="31">
         <f>SUM(I7:I18)</f>
@@ -6914,16 +6911,16 @@
     </row>
     <row r="6" ht="32.1" customHeight="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" s="32" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="C6" s="32" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="32" t="s">
-        <v>27</v>
-      </c>
       <c r="D6" s="32" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E6" s="32" t="s">
         <v>14</v>
@@ -6932,26 +6929,26 @@
         <v>16</v>
       </c>
       <c r="G6" s="32" t="s">
+        <v>27</v>
+      </c>
+      <c r="H6" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="H6" s="32" t="s">
+      <c r="I6" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="I6" s="32" t="s">
+      <c r="J6" s="32" t="s">
         <v>30</v>
       </c>
-      <c r="J6" s="32" t="s">
-        <v>31</v>
-      </c>
       <c r="L6" s="29" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M6" s="33">
         <f>IFERROR(M4/M3,0)</f>
         <v>0.6060606060606061</v>
       </c>
       <c r="N6" s="29" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="O6" s="33">
         <f>IFERROR(O4/O5,0)</f>

</xml_diff>